<commit_message>
chore(desktop): update sample files with realistic budget data
Add material fee, test fee, and external cooperation fee sheets
to sample xlsx and config to match real project budget structure.

Generated with [Claude Code](https://claude.ai/code)
via [Happy](https://happy.engineering)

Co-Authored-By: Claude <noreply@anthropic.com>
Co-Authored-By: Happy <yesreply@happy.engineering>
</commit_message>
<xml_diff>
--- a/apps/desktop/public/samples/sample-budget.xlsx
+++ b/apps/desktop/public/samples/sample-budget.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总页" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备费" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料费" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试费" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外部协作费" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,6 +126,96 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3810000" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3810000" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3810000" cy="1905000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,12 +507,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -440,7 +529,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150000</v>
+        <v>120000</v>
+      </c>
+      <c r="C2">
+        <f>B2+B3+B4+B5+B6</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -456,7 +549,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>测试化验加工费</t>
+          <t>测试费</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -476,12 +569,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B6">
-        <f>SUM(B2:B5)</f>
-        <v/>
+          <t>外部协作费</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>80000</v>
       </c>
     </row>
   </sheetData>
@@ -495,18 +587,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -553,16 +635,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>高性能工作站</t>
+          <t>高性能服务器</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CPU:i9-14900K / RAM:128GB / SSD:4TB</t>
+          <t>Dell R750</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>35000</v>
+        <v>50000</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -573,31 +655,31 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>项目计算需求，需高性能计算环境</t>
+          <t>计算需求</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>参考市场报价，单价约35000元</t>
+          <t>市场价格</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>便携式笔记本电脑</t>
+          <t>存储阵列</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CPU:i7-13700H / RAM:32GB / SSD:1TB</t>
+          <t>NetApp</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12000</v>
+        <v>20000</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E3">
         <f>C3*D3</f>
@@ -605,44 +687,331 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>项目组成员外出调研使用</t>
+          <t>数据存储</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>参考市场报价，单价约12000元</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>打印机</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>彩色激光/A3幅面/网络打印</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+          <t>厂商报价</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>规格</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>单价</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>经费</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>用途说明</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>采购依据</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>报价截图</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>试剂A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AR级</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>50</v>
+      </c>
+      <c r="E2">
+        <f>C2*D2</f>
+        <v/>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>实验用</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>批量采购</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>耗材B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>标准</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>500</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3">
+        <f>C3*D3</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>日常使用</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>协议价</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>规格</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>单价</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>经费</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>测试内容</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>计费依据</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>报价截图</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>性能测试</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>第三方</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>15000</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="E4">
-        <f>C4*D4</f>
+      <c r="E2">
+        <f>C2*D2</f>
         <v/>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>项目报告打印需求</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>参考市场报价，单价约15000元</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>系统验收</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>合同</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>安全测试</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>第三方</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <f>C3*D3</f>
+        <v/>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>合规要求</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>合同</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>经费</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>外协内容</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>计费依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>性能测试外包</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>委托第三方机构进行系统性能测试</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>按合同约定，一次性支付</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>安全评估</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>委托专业机构进行安全漏洞评估</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>按工作量计费</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(desktop): add HelpPopover, DropZone drag-drop, template batch operations, update sample files
- Add HelpPopover (?) to all pages with field descriptions
- Add DropZone component for drag-and-drop file import (Tauri onDragDropEvent)
- Fix HelpPopover overflow on right edge with auto-flip positioning
- Fix DropZone duplicate import by ensuring listener cleanup on unmount
- TemplateManager: add multi-select, select all, batch delete
- Update sample xlsx/config to match template Chinese placeholders
- Add sample images to equipment and materials sheets
- Bump version to 0.8.4

Generated with [Claude Code](https://claude.ai/code)
via [Happy](https://happy.engineering)

Co-Authored-By: Claude <noreply@anthropic.com>
Co-Authored-By: Happy <yesreply@happy.engineering>
</commit_message>
<xml_diff>
--- a/apps/desktop/public/samples/sample-budget.xlsx
+++ b/apps/desktop/public/samples/sample-budget.xlsx
@@ -10,8 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总页" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备费" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料费" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试费" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外部协作费" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="外部协作费" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="燃料动力费" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="会议差旅国际合作与交流费" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出版文献信息传播知识产权事务费" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="劳务费" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="专家咨询费" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="其他支出" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="间接经费" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,7 +143,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3810000" cy="1905000"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -145,6 +151,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1143000" cy="857250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -167,37 +198,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3810000" cy="1905000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="3810000" cy="1905000"/>
+    <ext cx="1143000" cy="857250"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -507,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,55 +526,278 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>设备费</t>
+          <t>直接费</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>120000</v>
-      </c>
-      <c r="C2">
-        <f>B2+B3+B4+B5+B6</f>
-        <v/>
+        <v>600000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>材料费</t>
+          <t>设备费</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>50000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>测试费</t>
+          <t>材料费</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>差旅费</t>
+          <t>外部协作费</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>外部协作费</t>
+          <t>燃料动力费</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80000</v>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>会议差旅国际合作交流费</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>出版文献信息传播知识产权事务费</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>劳务费</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>专家咨询费</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>其他支出</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>间接费用</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>管理费科研绩效支出</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>支出说明</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>测算依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>设备保险费</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>大型设备年度保险</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>保险费率估算</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>资料印刷费</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>研究报告印制</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>印刷厂报价</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>通讯网络费</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>项目专用通讯网络</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>运营商资费标准</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>金额（元）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>管理费</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>按直接费用比例提取</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>科研绩效支出</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>绩效奖励</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -587,8 +811,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -603,7 +830,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>单价</t>
+          <t>单价（元）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -613,7 +840,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>经费</t>
+          <t>经费（元）</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -640,27 +867,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Dell R750</t>
+          <t>Dell R750 / 128GB / 2×Xeon</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>50000</v>
+        <v>80000</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <f>C2*D2</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>80000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>计算需求</t>
+          <t>项目核心计算平台</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>市场价格</t>
+          <t>市场询价</t>
         </is>
       </c>
     </row>
@@ -672,27 +898,57 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NetApp</t>
+          <t>NetApp FAS2750 / 24TB</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3">
-        <f>C3*D3</f>
-        <v/>
+      <c r="E3" t="n">
+        <v>50000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>数据存储</t>
+          <t>科研数据存储</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>厂商报价</t>
+          <t>供应商报价</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>便携工作站</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ThinkPad P16 / 64GB</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>现场数据采集处理</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>官网价格</t>
         </is>
       </c>
     </row>
@@ -708,8 +964,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -724,7 +983,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>单价</t>
+          <t>单价（元）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -734,7 +993,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>经费</t>
+          <t>经费（元）</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -756,64 +1015,124 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>试剂A</t>
+          <t>实验试剂A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AR级</t>
+          <t>AR级 500mL</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
-      </c>
-      <c r="E2">
-        <f>C2*D2</f>
-        <v/>
+        <v>20</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>实验用</t>
+          <t>样品前处理</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>批量采购</t>
+          <t>实验室常用耗材</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>耗材B</t>
+          <t>色谱柱</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>标准</t>
+          <t>C18 250mm</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
-      </c>
-      <c r="E3">
-        <f>C3*D3</f>
-        <v/>
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>日常使用</t>
+          <t>液相色谱分析</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>协议价</t>
+          <t>品牌供应商</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>标准品</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>混合标液 100μg/mL</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>定量分析校准</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>国家标准物质中心</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>实验耗材</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>离心管/移液头等</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>日常实验消耗</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>市场采购</t>
         </is>
       </c>
     </row>
@@ -829,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -840,107 +1159,82 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>规格</t>
+          <t>经费（元）</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>单价</t>
+          <t>外协内容</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>数量</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>经费</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>测试内容</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>计费依据</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>报价截图</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>性能测试</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>第三方</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <f>C2*D2</f>
-        <v/>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>系统验收</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>合同</t>
+          <t>XX大学材料测试中心</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>材料微观结构表征</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>按样品计费</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>安全测试</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>第三方</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>15000</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <f>C3*D3</f>
-        <v/>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>合规要求</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>合同</t>
+          <t>YY检测技术有限公司</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>环境样品有害物质检测</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>检测项目单价×数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ZZ研究院</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>数据建模与仿真计算</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>人月费率×工作量</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -950,7 +1244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -961,57 +1255,531 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>经费</t>
+          <t>数量</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>外协内容</t>
+          <t>单价（元）</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>计费依据</t>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>用途说明</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>测算依据</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>性能测试外包</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>50000</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>委托第三方机构进行系统性能测试</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>按合同约定，一次性支付</t>
+          <t>电力消耗</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>实验室设备运行</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>历史用电数据</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>安全评估</t>
+          <t>水费</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12月</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>500</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>实验用水</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>市政水价估算</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>内容说明</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>计费依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>国内学术会议</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>参加年度学术研讨会</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>会议注册费+差旅</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>项目组出差</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30000</v>
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>外场试验与数据采集差旅</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>差旅标准×人次</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>国际学术交流</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>参加国际会议并报告</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>国际差旅标准</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>用途说明</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>计费依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>论文版面费</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SCI期刊论文发表</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>期刊收费标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>文献检索与数据库</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10000</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>委托专业机构进行安全漏洞评估</t>
+          <t>专业文献数据库使用费</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>按工作量计费</t>
+          <t>年度订阅费用</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>专利申请</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>发明专利申请2项</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>专利代理费+申请费</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>人数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>月数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>标准（元/月）</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>研究生助研津贴</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>72000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>博士/硕士研究生</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>临时劳务</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>36000</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>数据录入与整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>科研助理</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>实验室日常管理</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>人次</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>标准（元/次）</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>经费（元）</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>咨询内容</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>计费依据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>项目论证专家</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>项目立项论证评审</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>专家咨询费标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>技术咨询专家</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>关键技术方案咨询</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>专家咨询费标准</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>结题验收专家</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>项目结题验收评审</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>专家咨询费标准</t>
         </is>
       </c>
     </row>

</xml_diff>